<commit_message>
live update 01:40:10 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-zomb-emp2-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-zomb-emp2-2026-04-02_20260403_001542.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AD5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -739,6 +739,312 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>01:36:21</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.4854</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.2427</v>
+      </c>
+      <c r="J3" t="n">
+        <v>6200</v>
+      </c>
+      <c r="K3" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>4</v>
+      </c>
+      <c r="O3" t="n">
+        <v>5</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T3" s="2" t="n"/>
+      <c r="U3" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V3" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>01:37:55</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.6491</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.3246</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2800</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>9</v>
+      </c>
+      <c r="O4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T4" s="2" t="n"/>
+      <c r="U4" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V4" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>01:39:59</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0.7083</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.3542</v>
+      </c>
+      <c r="J5" t="n">
+        <v>7700</v>
+      </c>
+      <c r="K5" t="n">
+        <v>700</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>14</v>
+      </c>
+      <c r="O5" t="n">
+        <v>9</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>2</v>
+      </c>
+      <c r="R5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T5" s="2" t="n"/>
+      <c r="U5" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V5" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 01:45:12 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-zomb-emp2-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-zomb-emp2-2026-04-02_20260403_001542.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD5"/>
+  <dimension ref="A1:AD7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1045,6 +1045,210 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>01:45:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.7083</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.3542</v>
+      </c>
+      <c r="J6" t="n">
+        <v>7700</v>
+      </c>
+      <c r="K6" t="n">
+        <v>700</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>14</v>
+      </c>
+      <c r="O6" t="n">
+        <v>9</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>2</v>
+      </c>
+      <c r="R6" t="n">
+        <v>2</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T6" s="2" t="n"/>
+      <c r="U6" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V6" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>01:45:11</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0.5472</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0.2736</v>
+      </c>
+      <c r="J7" t="n">
+        <v>5900</v>
+      </c>
+      <c r="K7" t="n">
+        <v>3150</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>18</v>
+      </c>
+      <c r="O7" t="n">
+        <v>13</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>3</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T7" s="2" t="n"/>
+      <c r="U7" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V7" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 01:50:20 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-zomb-emp2-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-zomb-emp2-2026-04-02_20260403_001542.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD7"/>
+  <dimension ref="A1:AD15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1249,6 +1249,822 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>01:46:04</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0.5472</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.2736</v>
+      </c>
+      <c r="J8" t="n">
+        <v>5900</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3150</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>18</v>
+      </c>
+      <c r="O8" t="n">
+        <v>13</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>3</v>
+      </c>
+      <c r="R8" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T8" s="2" t="n"/>
+      <c r="U8" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V8" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>01:46:16</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0.7179</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0.3589</v>
+      </c>
+      <c r="J9" t="n">
+        <v>900</v>
+      </c>
+      <c r="K9" t="n">
+        <v>450</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>22</v>
+      </c>
+      <c r="O9" t="n">
+        <v>14</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>3</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T9" s="2" t="n"/>
+      <c r="U9" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V9" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>01:47:18</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0.7179</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0.3589</v>
+      </c>
+      <c r="J10" t="n">
+        <v>900</v>
+      </c>
+      <c r="K10" t="n">
+        <v>450</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>22</v>
+      </c>
+      <c r="O10" t="n">
+        <v>14</v>
+      </c>
+      <c r="P10" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T10" s="2" t="n"/>
+      <c r="U10" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V10" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>01:47:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0.7649</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0.3824</v>
+      </c>
+      <c r="J11" t="n">
+        <v>6150</v>
+      </c>
+      <c r="K11" t="n">
+        <v>850</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>27</v>
+      </c>
+      <c r="O11" t="n">
+        <v>17</v>
+      </c>
+      <c r="P11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>3</v>
+      </c>
+      <c r="R11" t="n">
+        <v>2</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T11" s="2" t="n"/>
+      <c r="U11" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V11" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>01:48:54</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>6-2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0.7649</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0.3824</v>
+      </c>
+      <c r="J12" t="n">
+        <v>6150</v>
+      </c>
+      <c r="K12" t="n">
+        <v>850</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>27</v>
+      </c>
+      <c r="O12" t="n">
+        <v>17</v>
+      </c>
+      <c r="P12" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R12" t="n">
+        <v>2</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T12" s="2" t="n"/>
+      <c r="U12" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V12" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>01:49:05</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>6-2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0.8485</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0.4243</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1150</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2850</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>32</v>
+      </c>
+      <c r="O13" t="n">
+        <v>17</v>
+      </c>
+      <c r="P13" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>3</v>
+      </c>
+      <c r="R13" t="n">
+        <v>3</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T13" s="2" t="n"/>
+      <c r="U13" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V13" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>01:49:58</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>9</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>7-2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0.8735000000000001</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0.4367</v>
+      </c>
+      <c r="J14" t="n">
+        <v>7350</v>
+      </c>
+      <c r="K14" t="n">
+        <v>4850</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>36</v>
+      </c>
+      <c r="O14" t="n">
+        <v>17</v>
+      </c>
+      <c r="P14" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>3</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T14" s="2" t="n"/>
+      <c r="U14" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V14" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>01:50:09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>9</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>7-2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0.8735000000000001</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0.4367</v>
+      </c>
+      <c r="J15" t="n">
+        <v>7350</v>
+      </c>
+      <c r="K15" t="n">
+        <v>4850</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>36</v>
+      </c>
+      <c r="O15" t="n">
+        <v>17</v>
+      </c>
+      <c r="P15" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" t="n">
+        <v>4</v>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T15" s="2" t="n"/>
+      <c r="U15" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V15" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 01:55:28 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-zomb-emp2-2026-04-02_20260403_001542.xlsx
+++ b/data/live_logs/live_cs2-zomb-emp2-2026-04-02_20260403_001542.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD15"/>
+  <dimension ref="A1:AD23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2065,6 +2065,822 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>01:51:23</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>9</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>7-3</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0.8735000000000001</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>0.4367</v>
+      </c>
+      <c r="J16" t="n">
+        <v>7350</v>
+      </c>
+      <c r="K16" t="n">
+        <v>4850</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>36</v>
+      </c>
+      <c r="O16" t="n">
+        <v>17</v>
+      </c>
+      <c r="P16" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>3</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4</v>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T16" s="2" t="n"/>
+      <c r="U16" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V16" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>01:51:34</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>7-3</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0.9146</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0.4573</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1100</v>
+      </c>
+      <c r="K17" t="n">
+        <v>7750</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>41</v>
+      </c>
+      <c r="O17" t="n">
+        <v>20</v>
+      </c>
+      <c r="P17" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>4</v>
+      </c>
+      <c r="R17" t="n">
+        <v>5</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T17" s="2" t="n"/>
+      <c r="U17" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V17" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>01:52:37</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>10</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>8-3</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0.9146</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0.4573</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1100</v>
+      </c>
+      <c r="K18" t="n">
+        <v>7750</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>41</v>
+      </c>
+      <c r="O18" t="n">
+        <v>20</v>
+      </c>
+      <c r="P18" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>4</v>
+      </c>
+      <c r="R18" t="n">
+        <v>5</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T18" s="2" t="n"/>
+      <c r="U18" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V18" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>01:52:48</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>11</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>8-3</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0.8933</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0.4466</v>
+      </c>
+      <c r="J19" t="n">
+        <v>2700</v>
+      </c>
+      <c r="K19" t="n">
+        <v>11750</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>43</v>
+      </c>
+      <c r="O19" t="n">
+        <v>25</v>
+      </c>
+      <c r="P19" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>5</v>
+      </c>
+      <c r="R19" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T19" s="2" t="n"/>
+      <c r="U19" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V19" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>01:54:02</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>11</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>9-3</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0.8933</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>0.4466</v>
+      </c>
+      <c r="J20" t="n">
+        <v>2700</v>
+      </c>
+      <c r="K20" t="n">
+        <v>11750</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>43</v>
+      </c>
+      <c r="O20" t="n">
+        <v>25</v>
+      </c>
+      <c r="P20" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>5</v>
+      </c>
+      <c r="R20" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T20" s="2" t="n"/>
+      <c r="U20" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V20" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>01:54:13</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>12</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>9-3</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>0.9182</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>0.4591</v>
+      </c>
+      <c r="J21" t="n">
+        <v>9200</v>
+      </c>
+      <c r="K21" t="n">
+        <v>2350</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>48</v>
+      </c>
+      <c r="O21" t="n">
+        <v>27</v>
+      </c>
+      <c r="P21" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>6</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T21" s="2" t="n"/>
+      <c r="U21" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V21" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>01:55:06</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>12</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>10-3</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0.9182</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>0.4591</v>
+      </c>
+      <c r="J22" t="n">
+        <v>9200</v>
+      </c>
+      <c r="K22" t="n">
+        <v>2350</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>48</v>
+      </c>
+      <c r="O22" t="n">
+        <v>27</v>
+      </c>
+      <c r="P22" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>6</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T22" s="2" t="n"/>
+      <c r="U22" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V22" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>01:55:17</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nuke</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>13</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>10-3</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>0.9363</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0.4681</v>
+      </c>
+      <c r="J23" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K23" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>53</v>
+      </c>
+      <c r="O23" t="n">
+        <v>31</v>
+      </c>
+      <c r="P23" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>6</v>
+      </c>
+      <c r="R23" t="n">
+        <v>2</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="T23" s="2" t="n"/>
+      <c r="U23" s="2" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="V23" t="n">
+        <v>15363.36891</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>WINNER:EMPIRE@0.001x50521; MAP2:Zomblers@0.001x37240; O/U:Under@0.001x38520</t>
+        </is>
+      </c>
+      <c r="Z23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>Zomblers LLC</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>Surge</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>